<commit_message>
Extend RADAR test datasets — add 20 kayak rows to ARG and RQ files
RADAR_Test_QMRA.xlsx already had 20 extra kayak rows (Site 1 & Site 2,
10 dates each) from a prior update that were causing 20 RADAR warnings
because they had no matching rows in the other two module files.

Added the same 20 (Site, Date) pairs to RADAR_Test_CAMRI_ARG.xlsx and
RADAR_Test_RQ.xlsx so all three files now match on all 220 pairs.
RADAR test run with all 3 files should produce 220 scored samples, 0 warnings.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dataset/RADAR_Test_CAMRI_ARG.xlsx
+++ b/docs/dataset/RADAR_Test_CAMRI_ARG.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -48,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P202"/>
+  <dimension ref="A1:P222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12553,6 +12555,1206 @@
         <v>819617.9</v>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240105</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="n">
+        <v>45296</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>90339.89999999999</v>
+      </c>
+      <c r="H203" t="n">
+        <v>950633.6</v>
+      </c>
+      <c r="I203" t="n">
+        <v>149971.1</v>
+      </c>
+      <c r="J203" t="n">
+        <v>739370.4</v>
+      </c>
+      <c r="K203" t="n">
+        <v>841242.4</v>
+      </c>
+      <c r="L203" t="n">
+        <v>747137</v>
+      </c>
+      <c r="M203" t="n">
+        <v>301937.6</v>
+      </c>
+      <c r="N203" t="n">
+        <v>351623.9</v>
+      </c>
+      <c r="O203" t="n">
+        <v>721862.6</v>
+      </c>
+      <c r="P203" t="n">
+        <v>965646.4</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240210</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="n">
+        <v>45332</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>662627.8</v>
+      </c>
+      <c r="H204" t="n">
+        <v>540581.2</v>
+      </c>
+      <c r="I204" t="n">
+        <v>387901.2</v>
+      </c>
+      <c r="J204" t="n">
+        <v>405739.7</v>
+      </c>
+      <c r="K204" t="n">
+        <v>719095.9</v>
+      </c>
+      <c r="L204" t="n">
+        <v>428891.2</v>
+      </c>
+      <c r="M204" t="n">
+        <v>534196.7</v>
+      </c>
+      <c r="N204" t="n">
+        <v>630948.6</v>
+      </c>
+      <c r="O204" t="n">
+        <v>632518.6</v>
+      </c>
+      <c r="P204" t="n">
+        <v>41025.8</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240317</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="n">
+        <v>45368</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>230611.6</v>
+      </c>
+      <c r="H205" t="n">
+        <v>705759.3</v>
+      </c>
+      <c r="I205" t="n">
+        <v>570348.3</v>
+      </c>
+      <c r="J205" t="n">
+        <v>837906.6</v>
+      </c>
+      <c r="K205" t="n">
+        <v>52486.3</v>
+      </c>
+      <c r="L205" t="n">
+        <v>231729.9</v>
+      </c>
+      <c r="M205" t="n">
+        <v>501970.6</v>
+      </c>
+      <c r="N205" t="n">
+        <v>746993.3</v>
+      </c>
+      <c r="O205" t="n">
+        <v>195089.1</v>
+      </c>
+      <c r="P205" t="n">
+        <v>764622.1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240422</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>410400.3</v>
+      </c>
+      <c r="H206" t="n">
+        <v>305663.7</v>
+      </c>
+      <c r="I206" t="n">
+        <v>829454.1</v>
+      </c>
+      <c r="J206" t="n">
+        <v>107128.4</v>
+      </c>
+      <c r="K206" t="n">
+        <v>933785.7</v>
+      </c>
+      <c r="L206" t="n">
+        <v>310524.5</v>
+      </c>
+      <c r="M206" t="n">
+        <v>362293.3</v>
+      </c>
+      <c r="N206" t="n">
+        <v>203077.5</v>
+      </c>
+      <c r="O206" t="n">
+        <v>467986.3</v>
+      </c>
+      <c r="P206" t="n">
+        <v>842275.2</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240528</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="n">
+        <v>45440</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>221066.8</v>
+      </c>
+      <c r="H207" t="n">
+        <v>554024.4</v>
+      </c>
+      <c r="I207" t="n">
+        <v>440223.9</v>
+      </c>
+      <c r="J207" t="n">
+        <v>301739.1</v>
+      </c>
+      <c r="K207" t="n">
+        <v>130187.5</v>
+      </c>
+      <c r="L207" t="n">
+        <v>697886</v>
+      </c>
+      <c r="M207" t="n">
+        <v>415113.9</v>
+      </c>
+      <c r="N207" t="n">
+        <v>469680.6</v>
+      </c>
+      <c r="O207" t="n">
+        <v>602678.7</v>
+      </c>
+      <c r="P207" t="n">
+        <v>106964.3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240703</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="n">
+        <v>45476</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>817723.1</v>
+      </c>
+      <c r="H208" t="n">
+        <v>890827.8</v>
+      </c>
+      <c r="I208" t="n">
+        <v>254308.3</v>
+      </c>
+      <c r="J208" t="n">
+        <v>816040.8</v>
+      </c>
+      <c r="K208" t="n">
+        <v>698841.6</v>
+      </c>
+      <c r="L208" t="n">
+        <v>298250.8</v>
+      </c>
+      <c r="M208" t="n">
+        <v>269845.5</v>
+      </c>
+      <c r="N208" t="n">
+        <v>83908.8</v>
+      </c>
+      <c r="O208" t="n">
+        <v>414151.7</v>
+      </c>
+      <c r="P208" t="n">
+        <v>451193.4</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240808</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="n">
+        <v>45512</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>486837</v>
+      </c>
+      <c r="H209" t="n">
+        <v>481530.4</v>
+      </c>
+      <c r="I209" t="n">
+        <v>548661.8</v>
+      </c>
+      <c r="J209" t="n">
+        <v>124791.8</v>
+      </c>
+      <c r="K209" t="n">
+        <v>224576.3</v>
+      </c>
+      <c r="L209" t="n">
+        <v>559146.4</v>
+      </c>
+      <c r="M209" t="n">
+        <v>472393.4</v>
+      </c>
+      <c r="N209" t="n">
+        <v>174386.8</v>
+      </c>
+      <c r="O209" t="n">
+        <v>276791.6</v>
+      </c>
+      <c r="P209" t="n">
+        <v>979108.3</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20240913</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>799013.9</v>
+      </c>
+      <c r="H210" t="n">
+        <v>726924.6</v>
+      </c>
+      <c r="I210" t="n">
+        <v>355285.8</v>
+      </c>
+      <c r="J210" t="n">
+        <v>418596.4</v>
+      </c>
+      <c r="K210" t="n">
+        <v>704907.2</v>
+      </c>
+      <c r="L210" t="n">
+        <v>561796.8</v>
+      </c>
+      <c r="M210" t="n">
+        <v>640474.6</v>
+      </c>
+      <c r="N210" t="n">
+        <v>35548.5</v>
+      </c>
+      <c r="O210" t="n">
+        <v>712577.4</v>
+      </c>
+      <c r="P210" t="n">
+        <v>200048</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20241019</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>October</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="n">
+        <v>45584</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>327461.1</v>
+      </c>
+      <c r="H211" t="n">
+        <v>530820.6</v>
+      </c>
+      <c r="I211" t="n">
+        <v>949190.1</v>
+      </c>
+      <c r="J211" t="n">
+        <v>405574.6</v>
+      </c>
+      <c r="K211" t="n">
+        <v>646121.4</v>
+      </c>
+      <c r="L211" t="n">
+        <v>208606.7</v>
+      </c>
+      <c r="M211" t="n">
+        <v>939503.5</v>
+      </c>
+      <c r="N211" t="n">
+        <v>247726.5</v>
+      </c>
+      <c r="O211" t="n">
+        <v>540846.2</v>
+      </c>
+      <c r="P211" t="n">
+        <v>680739.4</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>ARG-Site1-20241124</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Site 1</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="n">
+        <v>45620</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>699081.6</v>
+      </c>
+      <c r="H212" t="n">
+        <v>445444.2</v>
+      </c>
+      <c r="I212" t="n">
+        <v>647113.9</v>
+      </c>
+      <c r="J212" t="n">
+        <v>10242.6</v>
+      </c>
+      <c r="K212" t="n">
+        <v>985231.8</v>
+      </c>
+      <c r="L212" t="n">
+        <v>558351.7</v>
+      </c>
+      <c r="M212" t="n">
+        <v>595108.2</v>
+      </c>
+      <c r="N212" t="n">
+        <v>254383.2</v>
+      </c>
+      <c r="O212" t="n">
+        <v>480092.8</v>
+      </c>
+      <c r="P212" t="n">
+        <v>642499.2</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240123</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="n">
+        <v>45314</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>412454.9</v>
+      </c>
+      <c r="H213" t="n">
+        <v>121504.4</v>
+      </c>
+      <c r="I213" t="n">
+        <v>196400.9</v>
+      </c>
+      <c r="J213" t="n">
+        <v>873736.6</v>
+      </c>
+      <c r="K213" t="n">
+        <v>205660.8</v>
+      </c>
+      <c r="L213" t="n">
+        <v>514240.8</v>
+      </c>
+      <c r="M213" t="n">
+        <v>711082.6</v>
+      </c>
+      <c r="N213" t="n">
+        <v>221253.8</v>
+      </c>
+      <c r="O213" t="n">
+        <v>807758.2</v>
+      </c>
+      <c r="P213" t="n">
+        <v>475861.1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240228</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="n">
+        <v>45350</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>947073.3</v>
+      </c>
+      <c r="H214" t="n">
+        <v>204814</v>
+      </c>
+      <c r="I214" t="n">
+        <v>425344.6</v>
+      </c>
+      <c r="J214" t="n">
+        <v>362557.1</v>
+      </c>
+      <c r="K214" t="n">
+        <v>273086.4</v>
+      </c>
+      <c r="L214" t="n">
+        <v>426236.9</v>
+      </c>
+      <c r="M214" t="n">
+        <v>427086.5</v>
+      </c>
+      <c r="N214" t="n">
+        <v>394314.5</v>
+      </c>
+      <c r="O214" t="n">
+        <v>868121.7</v>
+      </c>
+      <c r="P214" t="n">
+        <v>325385.1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240404</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>56232.3</v>
+      </c>
+      <c r="H215" t="n">
+        <v>750133.7</v>
+      </c>
+      <c r="I215" t="n">
+        <v>434555.4</v>
+      </c>
+      <c r="J215" t="n">
+        <v>25075.7</v>
+      </c>
+      <c r="K215" t="n">
+        <v>754633.7</v>
+      </c>
+      <c r="L215" t="n">
+        <v>725979</v>
+      </c>
+      <c r="M215" t="n">
+        <v>654963.5</v>
+      </c>
+      <c r="N215" t="n">
+        <v>819742</v>
+      </c>
+      <c r="O215" t="n">
+        <v>269575.4</v>
+      </c>
+      <c r="P215" t="n">
+        <v>840454.8</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240510</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="n">
+        <v>45422</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G216" t="n">
+        <v>363789.2</v>
+      </c>
+      <c r="H216" t="n">
+        <v>859009.4</v>
+      </c>
+      <c r="I216" t="n">
+        <v>998563.1</v>
+      </c>
+      <c r="J216" t="n">
+        <v>554212.9</v>
+      </c>
+      <c r="K216" t="n">
+        <v>421798.6</v>
+      </c>
+      <c r="L216" t="n">
+        <v>734883.6</v>
+      </c>
+      <c r="M216" t="n">
+        <v>719454.2</v>
+      </c>
+      <c r="N216" t="n">
+        <v>505352.5</v>
+      </c>
+      <c r="O216" t="n">
+        <v>81358.39999999999</v>
+      </c>
+      <c r="P216" t="n">
+        <v>355683.7</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240615</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="n">
+        <v>45458</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G217" t="n">
+        <v>680481.6</v>
+      </c>
+      <c r="H217" t="n">
+        <v>13910.7</v>
+      </c>
+      <c r="I217" t="n">
+        <v>408962.9</v>
+      </c>
+      <c r="J217" t="n">
+        <v>916438.9</v>
+      </c>
+      <c r="K217" t="n">
+        <v>715072.2</v>
+      </c>
+      <c r="L217" t="n">
+        <v>260434.5</v>
+      </c>
+      <c r="M217" t="n">
+        <v>135826.6</v>
+      </c>
+      <c r="N217" t="n">
+        <v>571453.8</v>
+      </c>
+      <c r="O217" t="n">
+        <v>615149.8</v>
+      </c>
+      <c r="P217" t="n">
+        <v>286346.1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240721</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="n">
+        <v>45494</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G218" t="n">
+        <v>515835.5</v>
+      </c>
+      <c r="H218" t="n">
+        <v>991762.6</v>
+      </c>
+      <c r="I218" t="n">
+        <v>650113.3</v>
+      </c>
+      <c r="J218" t="n">
+        <v>542389.4</v>
+      </c>
+      <c r="K218" t="n">
+        <v>62536.3</v>
+      </c>
+      <c r="L218" t="n">
+        <v>474343.2</v>
+      </c>
+      <c r="M218" t="n">
+        <v>22487</v>
+      </c>
+      <c r="N218" t="n">
+        <v>963797.2</v>
+      </c>
+      <c r="O218" t="n">
+        <v>517056</v>
+      </c>
+      <c r="P218" t="n">
+        <v>600977.9</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20240826</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="n">
+        <v>45530</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>680683.4</v>
+      </c>
+      <c r="H219" t="n">
+        <v>40288.7</v>
+      </c>
+      <c r="I219" t="n">
+        <v>821415.4</v>
+      </c>
+      <c r="J219" t="n">
+        <v>698851.8</v>
+      </c>
+      <c r="K219" t="n">
+        <v>71943.7</v>
+      </c>
+      <c r="L219" t="n">
+        <v>914685.6</v>
+      </c>
+      <c r="M219" t="n">
+        <v>866031.9</v>
+      </c>
+      <c r="N219" t="n">
+        <v>990145.6</v>
+      </c>
+      <c r="O219" t="n">
+        <v>92570.10000000001</v>
+      </c>
+      <c r="P219" t="n">
+        <v>915692.2</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20241001</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>October</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="n">
+        <v>45566</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>779424.3</v>
+      </c>
+      <c r="H220" t="n">
+        <v>254241.3</v>
+      </c>
+      <c r="I220" t="n">
+        <v>79519.8</v>
+      </c>
+      <c r="J220" t="n">
+        <v>676551.2</v>
+      </c>
+      <c r="K220" t="n">
+        <v>62677.9</v>
+      </c>
+      <c r="L220" t="n">
+        <v>547651.2</v>
+      </c>
+      <c r="M220" t="n">
+        <v>805614.1</v>
+      </c>
+      <c r="N220" t="n">
+        <v>396437.3</v>
+      </c>
+      <c r="O220" t="n">
+        <v>332659</v>
+      </c>
+      <c r="P220" t="n">
+        <v>417091.7</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20241106</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="n">
+        <v>45602</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>114072.9</v>
+      </c>
+      <c r="H221" t="n">
+        <v>62317.6</v>
+      </c>
+      <c r="I221" t="n">
+        <v>564372.2</v>
+      </c>
+      <c r="J221" t="n">
+        <v>818568.8</v>
+      </c>
+      <c r="K221" t="n">
+        <v>991682.6</v>
+      </c>
+      <c r="L221" t="n">
+        <v>104095.9</v>
+      </c>
+      <c r="M221" t="n">
+        <v>303061</v>
+      </c>
+      <c r="N221" t="n">
+        <v>817119.4</v>
+      </c>
+      <c r="O221" t="n">
+        <v>291789.4</v>
+      </c>
+      <c r="P221" t="n">
+        <v>768144.6</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>ARG-Site2-20241212</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Site 2</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="n">
+        <v>45638</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="G222" t="n">
+        <v>940852.6</v>
+      </c>
+      <c r="H222" t="n">
+        <v>859090.9</v>
+      </c>
+      <c r="I222" t="n">
+        <v>624310.5</v>
+      </c>
+      <c r="J222" t="n">
+        <v>728439.7</v>
+      </c>
+      <c r="K222" t="n">
+        <v>857265.9</v>
+      </c>
+      <c r="L222" t="n">
+        <v>140951.5</v>
+      </c>
+      <c r="M222" t="n">
+        <v>336653.7</v>
+      </c>
+      <c r="N222" t="n">
+        <v>733919.9</v>
+      </c>
+      <c r="O222" t="n">
+        <v>477996.2</v>
+      </c>
+      <c r="P222" t="n">
+        <v>769338.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>